<commit_message>
add quan ly to hop va quan ly nganh
</commit_message>
<xml_diff>
--- a/docs/Chi tieu 2025.xlsx
+++ b/docs/Chi tieu 2025.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/caothanh/Library/CloudStorage/GoogleDrive-caominhthanh99@gmail.com/My Drive/DayHoc/XDPMPL/2026/project_tuyensinh/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1F01D1-0827-1046-BB49-D792C8806346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="29040" windowHeight="15720" tabRatio="447" xr2:uid="{356666A3-8437-8446-8021-A6A0316C3F1D}"/>
+    <workbookView windowWidth="23040" windowHeight="9000" tabRatio="447"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,9 +14,6 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -41,6 +32,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
   <si>
+    <t>DỰ KIẾN CHỈ TIÊU TUYỂN SINH NĂM 2025</t>
+  </si>
+  <si>
     <t>TT</t>
   </si>
   <si>
@@ -50,6 +44,9 @@
     <t>TÊN CTĐT</t>
   </si>
   <si>
+    <t>Chỉ tiêu chốt</t>
+  </si>
+  <si>
     <t>7140114</t>
   </si>
   <si>
@@ -137,9 +134,15 @@
     <t>7140247</t>
   </si>
   <si>
+    <t>Sư phạm Khoa học tự nhiên</t>
+  </si>
+  <si>
     <t>7140249</t>
   </si>
   <si>
+    <t>Sư phạm Lịch sử - Địa lý</t>
+  </si>
+  <si>
     <t>7220201</t>
   </si>
   <si>
@@ -311,6 +314,9 @@
     <t>7520207</t>
   </si>
   <si>
+    <t>Kỹ thuật điện tử - viễn thông (Thiết kế vi mạch)</t>
+  </si>
+  <si>
     <t>7810101</t>
   </si>
   <si>
@@ -324,45 +330,373 @@
   </si>
   <si>
     <t>* Các ngành đào tạo giáo viên đã ghi đúng chỉ tiêu đăng kí với Bộ GD&amp;ĐT</t>
-  </si>
-  <si>
-    <t>Chỉ tiêu chốt</t>
-  </si>
-  <si>
-    <t>Sư phạm Khoa học tự nhiên</t>
-  </si>
-  <si>
-    <t>Sư phạm Lịch sử - Địa lý</t>
-  </si>
-  <si>
-    <t>Kỹ thuật điện tử - viễn thông (Thiết kế vi mạch)</t>
-  </si>
-  <si>
-    <t>DỰ KIẾN CHỈ TIÊU TUYỂN SINH NĂM 2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="21">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -370,24 +704,310 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -436,7 +1056,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -469,26 +1089,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -521,23 +1124,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -699,716 +1285,712 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43024ACF-209E-3E48-A04B-4D5A2F3798A2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D52"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="16.1640625" customWidth="1"/>
-    <col min="3" max="3" width="50.6640625" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125"/>
+    <col min="2" max="2" width="16.1666666666667" customWidth="1"/>
+    <col min="3" max="3" width="50.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="10.8333333333333"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="B1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D3">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D4">
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D5">
         <v>200</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D6">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D7">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D8">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D9">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D10">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D11">
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4">
       <c r="A12">
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D12">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4">
       <c r="A13">
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D13">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4">
       <c r="A14">
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D14">
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4">
       <c r="A15">
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D15">
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D16">
         <v>120</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4">
       <c r="A17">
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="D17">
         <v>60</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4">
       <c r="A18">
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C18" t="s">
-        <v>97</v>
+        <v>36</v>
       </c>
       <c r="D18">
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4">
       <c r="A19">
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D19">
         <v>253</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4">
       <c r="A20">
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D20">
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4">
       <c r="A21">
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C21" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D21">
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4">
       <c r="A22">
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D22">
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4">
       <c r="A23">
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C23" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D23">
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4">
       <c r="A24">
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C24" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D24">
         <v>80</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4">
       <c r="A25">
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C25" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D25">
         <v>140</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4">
       <c r="A26">
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C26" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D26">
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4">
       <c r="A27">
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C27" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D27">
         <v>360</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4">
       <c r="A28">
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C28" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D28">
         <v>100</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4">
       <c r="A29">
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C29" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D29">
         <v>200</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4">
       <c r="A30">
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C30" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D30">
         <v>500</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4">
       <c r="A31">
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C31" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D31">
         <v>380</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4">
       <c r="A32">
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C32" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D32">
         <v>50</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4">
       <c r="A33">
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C33" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D33">
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4">
       <c r="A34">
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C34" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D34">
         <v>70</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4">
       <c r="A35">
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C35" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D35">
         <v>210</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4">
       <c r="A36">
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C36" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D36">
         <v>30</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4">
       <c r="A37">
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D37">
         <v>80</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4">
       <c r="A38">
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D38">
         <v>90</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4">
       <c r="A39">
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C39" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D39">
         <v>110</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4">
       <c r="A40">
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C40" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D40">
         <v>80</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4">
       <c r="A41">
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C41" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D41">
         <v>400</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4">
       <c r="A42">
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C42" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D42">
         <v>350</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4">
       <c r="A43">
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C43" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D43">
         <v>45</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4">
       <c r="A44">
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C44" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D44">
         <v>45</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4">
       <c r="A45">
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C45" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D45">
         <v>30</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4">
       <c r="A46">
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C46" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D46">
         <v>30</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C47" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D47">
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C48" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D48">
         <v>120</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C49" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D49">
         <v>60</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:4">
       <c r="D50">
         <f>SUM(D3:D49)</f>
         <v>5213</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:4">
       <c r="B52" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>